<commit_message>
Ajouter le Multitool-M4 (1er prix national) et corriger les points de l'audit
- Nouvelle page projet Multitool-M4 : dossier, code source des deux cartes, photos
- Accueil, Projets, sitemap et tableau de synthèse mis à jour
- Pages projet : section « Points techniques », vraies images sur les cartes
- Compétences, veille, stages : contenus corrigés, stage de 2ème année masqué
- Accessibilité : icônes décoratives masquées, contraste des badges, onglet actif
- Styles inline regroupés en classes, polices et dimensions d'images homogènes
- Netlify : iframes du site autorisées, Content-Security-Policy ajoutée
- Tableau de synthèse Excel : option SLAM, périodes, croix, stage NEPTING
- Dépôt : dossiers .idea et images NaniChat inutilisées retirés

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Tableau_de_synthese.xlsx
+++ b/Tableau_de_synthese.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="50">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -89,7 +89,7 @@
     <t>▢ SISR</t>
   </si>
   <si>
-    <t>▢ SLAM</t>
+    <t>☒ SLAM</t>
   </si>
   <si>
     <t xml:space="preserve">Réalisation en cours de formation
@@ -162,6 +162,36 @@
   </si>
   <si>
     <t>SESSION 2027</t>
+  </si>
+  <si>
+    <t>Workshop 2ème année - Projet Multitool-M4 (1er prix national).</t>
+  </si>
+  <si>
+    <t>Septembre 2026</t>
+  </si>
+  <si>
+    <t>du 15/09/25 au 19/09/25</t>
+  </si>
+  <si>
+    <t>du 01/11/25 au 31/12/25</t>
+  </si>
+  <si>
+    <t>du 01/01/26 au 28/02/26</t>
+  </si>
+  <si>
+    <t>du 01/10/25 au 30/11/25</t>
+  </si>
+  <si>
+    <t>du 01/10/25 au 31/12/25</t>
+  </si>
+  <si>
+    <t>du 14/09/26 au 18/09/26</t>
+  </si>
+  <si>
+    <t>Stage NEPTING - Développement d'outils de test monétiques (Java / Android).</t>
+  </si>
+  <si>
+    <t>du 20/04/26 au 29/05/26</t>
   </si>
 </sst>
 </file>
@@ -1394,26 +1424,16 @@
         <v>25</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="E9" s="16" t="s">
-        <v>28</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="C9" s="16"/>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
       <c r="F9" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="G9" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="H9" s="22" t="s">
-        <v>28</v>
-      </c>
+      <c r="G9" s="16"/>
+      <c r="H9" s="22"/>
       <c r="I9"/>
       <c r="J9"/>
       <c r="K9"/>
@@ -1512,7 +1532,7 @@
         <v>34</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="C11" s="16" t="s">
         <v>28</v>
@@ -1523,15 +1543,11 @@
       <c r="E11" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="F11" s="16" t="s">
-        <v>28</v>
-      </c>
+      <c r="F11" s="16"/>
       <c r="G11" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="H11" s="22" t="s">
-        <v>28</v>
-      </c>
+      <c r="H11" s="22"/>
       <c r="I11"/>
       <c r="J11"/>
       <c r="K11"/>
@@ -1573,7 +1589,7 @@
         <v>35</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="C12" s="16" t="s">
         <v>28</v>
@@ -1581,18 +1597,14 @@
       <c r="D12" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="16" t="s">
-        <v>28</v>
-      </c>
+      <c r="E12" s="16"/>
       <c r="F12" s="16" t="s">
         <v>28</v>
       </c>
       <c r="G12" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="H12" s="22" t="s">
-        <v>28</v>
-      </c>
+      <c r="H12" s="22"/>
       <c r="I12"/>
       <c r="J12"/>
       <c r="K12"/>
@@ -1634,26 +1646,20 @@
         <v>36</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="C13" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="16" t="s">
-        <v>28</v>
-      </c>
+      <c r="D13" s="16"/>
       <c r="E13" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="F13" s="16" t="s">
-        <v>28</v>
-      </c>
+      <c r="F13" s="16"/>
       <c r="G13" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="H13" s="22" t="s">
-        <v>28</v>
-      </c>
+      <c r="H13" s="22"/>
       <c r="I13"/>
       <c r="J13"/>
       <c r="K13"/>
@@ -1695,26 +1701,18 @@
         <v>37</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>28</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C14" s="16"/>
       <c r="D14" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="16" t="s">
-        <v>28</v>
-      </c>
-      <c r="F14" s="16" t="s">
-        <v>28</v>
-      </c>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
       <c r="G14" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="H14" s="22" t="s">
-        <v>28</v>
-      </c>
+      <c r="H14" s="22"/>
       <c r="I14"/>
       <c r="J14"/>
       <c r="K14"/>
@@ -1752,13 +1750,21 @@
       <c r="AQ14"/>
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A15" s="11"/>
-      <c r="B15" s="10"/>
+      <c r="A15" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>47</v>
+      </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-      <c r="G15" s="16"/>
+      <c r="F15" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="G15" s="16" t="s">
+        <v>28</v>
+      </c>
       <c r="H15" s="22"/>
       <c r="I15"/>
       <c r="J15"/>
@@ -1979,14 +1985,26 @@
       <c r="AQ19"/>
     </row>
     <row r="20" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A20" s="11"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="16"/>
-      <c r="D20" s="16"/>
+      <c r="A20" s="11" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D20" s="16" t="s">
+        <v>28</v>
+      </c>
       <c r="E20" s="16"/>
       <c r="F20" s="16"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="22"/>
+      <c r="G20" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="H20" s="22" t="s">
+        <v>28</v>
+      </c>
       <c r="I20"/>
       <c r="J20"/>
       <c r="K20"/>

</xml_diff>